<commit_message>
clean upto script 3
</commit_message>
<xml_diff>
--- a/closed_loan_backfill/source_sheets/CLOSED_LOAN_TRACKER.xlsx
+++ b/closed_loan_backfill/source_sheets/CLOSED_LOAN_TRACKER.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19626" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20106" uniqueCount="1010">
   <si>
     <t>Application No.</t>
   </si>
@@ -2845,6 +2845,353 @@
   </si>
   <si>
     <t>STTL48202411010135</t>
+  </si>
+  <si>
+    <t>INEVYF5110500264</t>
+  </si>
+  <si>
+    <t>STTL48202411050310</t>
+  </si>
+  <si>
+    <t>UPI- 390979257125</t>
+  </si>
+  <si>
+    <t>INEVYE5110500540</t>
+  </si>
+  <si>
+    <t>STTL48202411050933</t>
+  </si>
+  <si>
+    <t>Cash collected by Neeraj and UPI- 519622287134</t>
+  </si>
+  <si>
+    <t>CLN2704EV51212512FG00513</t>
+  </si>
+  <si>
+    <t>STTL48202502080491</t>
+  </si>
+  <si>
+    <t>INEVYG5110500336</t>
+  </si>
+  <si>
+    <t>STTL48202505271086</t>
+  </si>
+  <si>
+    <t>Shekhar</t>
+  </si>
+  <si>
+    <t>Cash Collected by Shekhar</t>
+  </si>
+  <si>
+    <t>INEVYG5110500297</t>
+  </si>
+  <si>
+    <t>STTL48202505271127</t>
+  </si>
+  <si>
+    <t>INEVYG5110500314</t>
+  </si>
+  <si>
+    <t>STTL48202505271554</t>
+  </si>
+  <si>
+    <t>INEVYG5110500316</t>
+  </si>
+  <si>
+    <t>STTL48202505271322</t>
+  </si>
+  <si>
+    <t>INRTYH5110501947</t>
+  </si>
+  <si>
+    <t>STTL48202507251064</t>
+  </si>
+  <si>
+    <t>Cash recceived by Neeraj
+UPI- 530581664726</t>
+  </si>
+  <si>
+    <t>INGFYJ5113200143</t>
+  </si>
+  <si>
+    <t>STTL48202507252806</t>
+  </si>
+  <si>
+    <t>INRTYJ5110501556</t>
+  </si>
+  <si>
+    <t>STTL48202507253022</t>
+  </si>
+  <si>
+    <t>INRTYJ5110501547</t>
+  </si>
+  <si>
+    <t>STTL48202507255977</t>
+  </si>
+  <si>
+    <t>Nischalanand</t>
+  </si>
+  <si>
+    <t>Cash received by Nischalanand</t>
+  </si>
+  <si>
+    <t>INRTYK5110501232</t>
+  </si>
+  <si>
+    <t>STTL48202507255429</t>
+  </si>
+  <si>
+    <t>INRTYK5110501136</t>
+  </si>
+  <si>
+    <t>STTL48202507254915</t>
+  </si>
+  <si>
+    <t>INRTYK5110501397</t>
+  </si>
+  <si>
+    <t>STTL48202505272447</t>
+  </si>
+  <si>
+    <t>INRTYL5110500481</t>
+  </si>
+  <si>
+    <t>CQ-2371</t>
+  </si>
+  <si>
+    <t>INEVYD5110500674</t>
+  </si>
+  <si>
+    <t>3D91A0002313355</t>
+  </si>
+  <si>
+    <t>Customer Requested for EMI to be on 13th</t>
+  </si>
+  <si>
+    <t>INEVYD5110500655</t>
+  </si>
+  <si>
+    <t>3D91A0002313349</t>
+  </si>
+  <si>
+    <t>UPI - 509225873156</t>
+  </si>
+  <si>
+    <t>INEVYE5110500486</t>
+  </si>
+  <si>
+    <t>STTL48202411010022</t>
+  </si>
+  <si>
+    <t>CLN2702EV51210517FG10496</t>
+  </si>
+  <si>
+    <t>STTL48202502080769</t>
+  </si>
+  <si>
+    <t>CLN2702EV51210517FG10495</t>
+  </si>
+  <si>
+    <t>STTL48202502080771</t>
+  </si>
+  <si>
+    <t>CLN2751EV51210008HG13734</t>
+  </si>
+  <si>
+    <t>STTL48202505273301</t>
+  </si>
+  <si>
+    <t>Hukam Singh Rathore</t>
+  </si>
+  <si>
+    <t>CLN2751EV51210008HG13759</t>
+  </si>
+  <si>
+    <t>STTL48202505273319</t>
+  </si>
+  <si>
+    <t>CLN2751EV51210008HG13747</t>
+  </si>
+  <si>
+    <t>STTL48202505273444</t>
+  </si>
+  <si>
+    <t>CLN2768EV51210508IG16164</t>
+  </si>
+  <si>
+    <t>STTL48202507253049</t>
+  </si>
+  <si>
+    <t>UPI- 300094777362</t>
+  </si>
+  <si>
+    <t>CLN2768EV51210508IG16177</t>
+  </si>
+  <si>
+    <t>STTL48202507253019</t>
+  </si>
+  <si>
+    <t>Mohd Azhar</t>
+  </si>
+  <si>
+    <t>CLN2771EV51210522IG17263</t>
+  </si>
+  <si>
+    <t>STTL48202507253112</t>
+  </si>
+  <si>
+    <t>Khushiram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash receievd by Khushiram 15,000 &amp;
+old e-rikshaw of 10,000 </t>
+  </si>
+  <si>
+    <t>INRTYJ5110501499</t>
+  </si>
+  <si>
+    <t>CQ-1242</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>Cash received by Yogesh</t>
+  </si>
+  <si>
+    <t>CLN2789EV51210501KG19670</t>
+  </si>
+  <si>
+    <t>CQ-1227</t>
+  </si>
+  <si>
+    <t>CLN2789EV51210501KG19654</t>
+  </si>
+  <si>
+    <t>CQ-1449</t>
+  </si>
+  <si>
+    <t>INRTYJ5110501478</t>
+  </si>
+  <si>
+    <t>STTL48202507255434</t>
+  </si>
+  <si>
+    <t>CLN2789EV51210501KG19661</t>
+  </si>
+  <si>
+    <t>CQ-1712</t>
+  </si>
+  <si>
+    <t>Diwker</t>
+  </si>
+  <si>
+    <t>CLN2539EV60810020BG00187</t>
+  </si>
+  <si>
+    <t>4B91A0002312083</t>
+  </si>
+  <si>
+    <t>Cash received by Shivam Bhati
+UPI - 521647052082</t>
+  </si>
+  <si>
+    <t>INEVYG5110500368</t>
+  </si>
+  <si>
+    <t>CQ-28</t>
+  </si>
+  <si>
+    <t>Cash received by Shivam Bhati,
+UPI 110364772821</t>
+  </si>
+  <si>
+    <t>INRTYH5110500980</t>
+  </si>
+  <si>
+    <t>STTL48202505272963</t>
+  </si>
+  <si>
+    <t>12000</t>
+  </si>
+  <si>
+    <t>Battrey Received By Shivam</t>
+  </si>
+  <si>
+    <t>INRTYH5110501709</t>
+  </si>
+  <si>
+    <t>STTL48202411050250</t>
+  </si>
+  <si>
+    <t>INRTYI5110502275</t>
+  </si>
+  <si>
+    <t>STTL48202507251043</t>
+  </si>
+  <si>
+    <t>khushi</t>
+  </si>
+  <si>
+    <t>5000 Cash Received by Khushi on 16/10/2025 
+13000 Cash received by Khushi Gill On 17/10/2025</t>
+  </si>
+  <si>
+    <t>CLN2771EV51210522IG17272</t>
+  </si>
+  <si>
+    <t>STTL48202507251301</t>
+  </si>
+  <si>
+    <t>UPI 933078033788</t>
+  </si>
+  <si>
+    <t>INRTYJ5110500892</t>
+  </si>
+  <si>
+    <t>STTL48202507253288</t>
+  </si>
+  <si>
+    <t>INRTYJ5110501471</t>
+  </si>
+  <si>
+    <t>STTL48202507252187</t>
+  </si>
+  <si>
+    <t>INRTYI5110502232</t>
+  </si>
+  <si>
+    <t>STTL48202507253236</t>
+  </si>
+  <si>
+    <t>Cash received By Mukul</t>
+  </si>
+  <si>
+    <t>CLN2789EV51210510KG20215</t>
+  </si>
+  <si>
+    <t>CQ-871</t>
+  </si>
+  <si>
+    <t>CLN2824EV51210504LG21746</t>
+  </si>
+  <si>
+    <t>CQ-1922</t>
+  </si>
+  <si>
+    <t>UPI 535190758692</t>
+  </si>
+  <si>
+    <t>INRTYK5110500667</t>
+  </si>
+  <si>
+    <t>STTL48202507255045</t>
+  </si>
+  <si>
+    <t>INRTYL5110500638</t>
+  </si>
+  <si>
+    <t>STTL48202507252192</t>
   </si>
 </sst>
 </file>
@@ -3423,6 +3770,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="6" width="12.63"/>
+    <col customWidth="1" min="20" max="20" width="18.38"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -76509,6 +76857,3884 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="62">
+        <v>54.0</v>
+      </c>
+      <c r="B85" s="63" t="s">
+        <v>123</v>
+      </c>
+      <c r="C85" s="64">
+        <v>45822.0</v>
+      </c>
+      <c r="D85" s="63" t="s">
+        <v>124</v>
+      </c>
+      <c r="E85" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F85" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G85" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H85" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I85" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J85" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K85" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L85" s="64">
+        <v>45822.0</v>
+      </c>
+      <c r="M85" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N85" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O85" s="66"/>
+      <c r="P85" s="67"/>
+      <c r="Q85" s="67"/>
+      <c r="R85" s="66"/>
+      <c r="S85" s="67"/>
+      <c r="T85" s="67"/>
+      <c r="U85" s="66"/>
+      <c r="V85" s="67"/>
+      <c r="W85" s="67"/>
+      <c r="X85" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y85" s="63" t="s">
+        <v>554</v>
+      </c>
+      <c r="Z85" s="63" t="s">
+        <v>872</v>
+      </c>
+      <c r="AA85" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB85" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC85" s="63" t="s">
+        <v>896</v>
+      </c>
+      <c r="AD85" s="63" t="s">
+        <v>897</v>
+      </c>
+      <c r="AE85" s="63">
+        <v>8.528963857E9</v>
+      </c>
+      <c r="AF85" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG85" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH85" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI85" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="62">
+        <v>77.0</v>
+      </c>
+      <c r="B86" s="63" t="s">
+        <v>141</v>
+      </c>
+      <c r="C86" s="64">
+        <v>45831.0</v>
+      </c>
+      <c r="D86" s="63" t="s">
+        <v>142</v>
+      </c>
+      <c r="E86" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F86" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G86" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H86" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="I86" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J86" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K86" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L86" s="64">
+        <v>45831.0</v>
+      </c>
+      <c r="M86" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N86" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="O86" s="66"/>
+      <c r="P86" s="67"/>
+      <c r="Q86" s="67"/>
+      <c r="R86" s="66"/>
+      <c r="S86" s="67"/>
+      <c r="T86" s="67"/>
+      <c r="U86" s="66"/>
+      <c r="V86" s="67"/>
+      <c r="W86" s="67"/>
+      <c r="X86" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y86" s="63" t="s">
+        <v>727</v>
+      </c>
+      <c r="Z86" s="63" t="s">
+        <v>898</v>
+      </c>
+      <c r="AA86" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB86" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC86" s="63" t="s">
+        <v>899</v>
+      </c>
+      <c r="AD86" s="63" t="s">
+        <v>900</v>
+      </c>
+      <c r="AE86" s="63">
+        <v>7.607970966E9</v>
+      </c>
+      <c r="AF86" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG86" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH86" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI86" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="62">
+        <v>125.0</v>
+      </c>
+      <c r="B87" s="63" t="s">
+        <v>158</v>
+      </c>
+      <c r="C87" s="64">
+        <v>45853.0</v>
+      </c>
+      <c r="D87" s="63" t="s">
+        <v>159</v>
+      </c>
+      <c r="E87" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F87" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G87" s="62">
+        <v>11190.0</v>
+      </c>
+      <c r="H87" s="62">
+        <v>810.0</v>
+      </c>
+      <c r="I87" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J87" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K87" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L87" s="64">
+        <v>45853.0</v>
+      </c>
+      <c r="M87" s="63">
+        <v>11190.0</v>
+      </c>
+      <c r="N87" s="63">
+        <v>810.0</v>
+      </c>
+      <c r="O87" s="66"/>
+      <c r="P87" s="67"/>
+      <c r="Q87" s="67"/>
+      <c r="R87" s="66"/>
+      <c r="S87" s="67"/>
+      <c r="T87" s="67"/>
+      <c r="U87" s="66"/>
+      <c r="V87" s="67"/>
+      <c r="W87" s="67"/>
+      <c r="X87" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y87" s="63" t="s">
+        <v>741</v>
+      </c>
+      <c r="Z87" s="63" t="s">
+        <v>901</v>
+      </c>
+      <c r="AA87" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB87" s="62">
+        <v>4000.0</v>
+      </c>
+      <c r="AC87" s="63" t="s">
+        <v>902</v>
+      </c>
+      <c r="AD87" s="63" t="s">
+        <v>903</v>
+      </c>
+      <c r="AE87" s="63">
+        <v>9.519060972E9</v>
+      </c>
+      <c r="AF87" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG87" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH87" s="65" t="s">
+        <v>776</v>
+      </c>
+      <c r="AI87" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="62">
+        <v>156.0</v>
+      </c>
+      <c r="B88" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="C88" s="64">
+        <v>45863.0</v>
+      </c>
+      <c r="D88" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="E88" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F88" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G88" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H88" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I88" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J88" s="73"/>
+      <c r="K88" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L88" s="64">
+        <v>45863.0</v>
+      </c>
+      <c r="M88" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N88" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O88" s="66"/>
+      <c r="P88" s="67"/>
+      <c r="Q88" s="67"/>
+      <c r="R88" s="66"/>
+      <c r="S88" s="67"/>
+      <c r="T88" s="67"/>
+      <c r="U88" s="66"/>
+      <c r="V88" s="67"/>
+      <c r="W88" s="67"/>
+      <c r="X88" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y88" s="63" t="s">
+        <v>780</v>
+      </c>
+      <c r="Z88" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA88" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB88" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC88" s="63" t="s">
+        <v>904</v>
+      </c>
+      <c r="AD88" s="63" t="s">
+        <v>905</v>
+      </c>
+      <c r="AE88" s="63">
+        <v>8.528183934E9</v>
+      </c>
+      <c r="AF88" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG88" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH88" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI88" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="62">
+        <v>171.0</v>
+      </c>
+      <c r="B89" s="63" t="s">
+        <v>172</v>
+      </c>
+      <c r="C89" s="64">
+        <v>45869.0</v>
+      </c>
+      <c r="D89" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="E89" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F89" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G89" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H89" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I89" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J89" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K89" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L89" s="64">
+        <v>45869.0</v>
+      </c>
+      <c r="M89" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N89" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O89" s="66"/>
+      <c r="P89" s="67"/>
+      <c r="Q89" s="67"/>
+      <c r="R89" s="66"/>
+      <c r="S89" s="67"/>
+      <c r="T89" s="67"/>
+      <c r="U89" s="66"/>
+      <c r="V89" s="67"/>
+      <c r="W89" s="67"/>
+      <c r="X89" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y89" s="63" t="s">
+        <v>906</v>
+      </c>
+      <c r="Z89" s="63" t="s">
+        <v>907</v>
+      </c>
+      <c r="AA89" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB89" s="62">
+        <v>3600.0</v>
+      </c>
+      <c r="AC89" s="63" t="s">
+        <v>908</v>
+      </c>
+      <c r="AD89" s="63" t="s">
+        <v>909</v>
+      </c>
+      <c r="AE89" s="63">
+        <v>6.306252861E9</v>
+      </c>
+      <c r="AF89" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG89" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH89" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI89" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="62">
+        <v>196.0</v>
+      </c>
+      <c r="B90" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="C90" s="64">
+        <v>45879.0</v>
+      </c>
+      <c r="D90" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="E90" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F90" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G90" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H90" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I90" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J90" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K90" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L90" s="64">
+        <v>45879.0</v>
+      </c>
+      <c r="M90" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N90" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O90" s="66"/>
+      <c r="P90" s="67"/>
+      <c r="Q90" s="67"/>
+      <c r="R90" s="66"/>
+      <c r="S90" s="67"/>
+      <c r="T90" s="67"/>
+      <c r="U90" s="66"/>
+      <c r="V90" s="67"/>
+      <c r="W90" s="67"/>
+      <c r="X90" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y90" s="63" t="s">
+        <v>732</v>
+      </c>
+      <c r="Z90" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA90" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB90" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC90" s="63" t="s">
+        <v>910</v>
+      </c>
+      <c r="AD90" s="63" t="s">
+        <v>911</v>
+      </c>
+      <c r="AE90" s="63">
+        <v>8.115994039E9</v>
+      </c>
+      <c r="AF90" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG90" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH90" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI90" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="62">
+        <v>198.0</v>
+      </c>
+      <c r="B91" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="C91" s="64">
+        <v>45881.0</v>
+      </c>
+      <c r="D91" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="E91" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F91" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G91" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H91" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I91" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J91" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K91" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L91" s="64">
+        <v>45881.0</v>
+      </c>
+      <c r="M91" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N91" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O91" s="66"/>
+      <c r="P91" s="67"/>
+      <c r="Q91" s="67"/>
+      <c r="R91" s="66"/>
+      <c r="S91" s="67"/>
+      <c r="T91" s="67"/>
+      <c r="U91" s="66"/>
+      <c r="V91" s="67"/>
+      <c r="W91" s="67"/>
+      <c r="X91" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y91" s="63" t="s">
+        <v>732</v>
+      </c>
+      <c r="Z91" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA91" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB91" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC91" s="63" t="s">
+        <v>912</v>
+      </c>
+      <c r="AD91" s="63" t="s">
+        <v>913</v>
+      </c>
+      <c r="AE91" s="63">
+        <v>9.140162787E9</v>
+      </c>
+      <c r="AF91" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG91" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH91" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI91" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="62">
+        <v>325.0</v>
+      </c>
+      <c r="B92" s="63" t="s">
+        <v>231</v>
+      </c>
+      <c r="C92" s="64">
+        <v>45923.0</v>
+      </c>
+      <c r="D92" s="63" t="s">
+        <v>232</v>
+      </c>
+      <c r="E92" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F92" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G92" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H92" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I92" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J92" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K92" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L92" s="64">
+        <v>45923.0</v>
+      </c>
+      <c r="M92" s="63">
+        <v>8000.0</v>
+      </c>
+      <c r="N92" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O92" s="66"/>
+      <c r="P92" s="67"/>
+      <c r="Q92" s="67"/>
+      <c r="R92" s="66"/>
+      <c r="S92" s="67"/>
+      <c r="T92" s="67"/>
+      <c r="U92" s="66"/>
+      <c r="V92" s="67"/>
+      <c r="W92" s="67"/>
+      <c r="X92" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y92" s="63" t="s">
+        <v>732</v>
+      </c>
+      <c r="Z92" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA92" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB92" s="62">
+        <v>4500.0</v>
+      </c>
+      <c r="AC92" s="63" t="s">
+        <v>914</v>
+      </c>
+      <c r="AD92" s="63" t="s">
+        <v>915</v>
+      </c>
+      <c r="AE92" s="63">
+        <v>8.429739615E9</v>
+      </c>
+      <c r="AF92" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG92" s="62">
+        <v>15.0</v>
+      </c>
+      <c r="AH92" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI92" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="62">
+        <v>478.0</v>
+      </c>
+      <c r="B93" s="63" t="s">
+        <v>248</v>
+      </c>
+      <c r="C93" s="64">
+        <v>45962.0</v>
+      </c>
+      <c r="D93" s="63" t="s">
+        <v>249</v>
+      </c>
+      <c r="E93" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F93" s="62">
+        <v>30000.0</v>
+      </c>
+      <c r="G93" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="H93" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="I93" s="62">
+        <v>30000.0</v>
+      </c>
+      <c r="J93" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K93" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L93" s="64">
+        <v>45962.0</v>
+      </c>
+      <c r="M93" s="63">
+        <v>15000.0</v>
+      </c>
+      <c r="N93" s="63">
+        <v>15000.0</v>
+      </c>
+      <c r="O93" s="66"/>
+      <c r="P93" s="67"/>
+      <c r="Q93" s="67"/>
+      <c r="R93" s="66"/>
+      <c r="S93" s="67"/>
+      <c r="T93" s="67"/>
+      <c r="U93" s="66"/>
+      <c r="V93" s="67"/>
+      <c r="W93" s="67"/>
+      <c r="X93" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y93" s="63" t="s">
+        <v>741</v>
+      </c>
+      <c r="Z93" s="63" t="s">
+        <v>916</v>
+      </c>
+      <c r="AA93" s="62">
+        <v>30000.0</v>
+      </c>
+      <c r="AB93" s="62">
+        <v>4160.0</v>
+      </c>
+      <c r="AC93" s="63" t="s">
+        <v>917</v>
+      </c>
+      <c r="AD93" s="63" t="s">
+        <v>918</v>
+      </c>
+      <c r="AE93" s="63">
+        <v>6.280722964E9</v>
+      </c>
+      <c r="AF93" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG93" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH93" s="65" t="s">
+        <v>776</v>
+      </c>
+      <c r="AI93" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="62">
+        <v>520.0</v>
+      </c>
+      <c r="B94" s="63" t="s">
+        <v>266</v>
+      </c>
+      <c r="C94" s="64">
+        <v>45974.0</v>
+      </c>
+      <c r="D94" s="63" t="s">
+        <v>267</v>
+      </c>
+      <c r="E94" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F94" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G94" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H94" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I94" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J94" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K94" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L94" s="64">
+        <v>45974.0</v>
+      </c>
+      <c r="M94" s="63">
+        <v>8000.0</v>
+      </c>
+      <c r="N94" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O94" s="66"/>
+      <c r="P94" s="67"/>
+      <c r="Q94" s="67"/>
+      <c r="R94" s="66"/>
+      <c r="S94" s="67"/>
+      <c r="T94" s="67"/>
+      <c r="U94" s="66"/>
+      <c r="V94" s="67"/>
+      <c r="W94" s="67"/>
+      <c r="X94" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y94" s="63" t="s">
+        <v>729</v>
+      </c>
+      <c r="Z94" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA94" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB94" s="62">
+        <v>7900.0</v>
+      </c>
+      <c r="AC94" s="63" t="s">
+        <v>919</v>
+      </c>
+      <c r="AD94" s="63" t="s">
+        <v>920</v>
+      </c>
+      <c r="AE94" s="63">
+        <v>7.977498177E9</v>
+      </c>
+      <c r="AF94" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG94" s="62">
+        <v>8.0</v>
+      </c>
+      <c r="AH94" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI94" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="62">
+        <v>640.0</v>
+      </c>
+      <c r="B95" s="63" t="s">
+        <v>276</v>
+      </c>
+      <c r="C95" s="64">
+        <v>45995.0</v>
+      </c>
+      <c r="D95" s="63" t="s">
+        <v>277</v>
+      </c>
+      <c r="E95" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F95" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="G95" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="H95" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I95" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="J95" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K95" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L95" s="64">
+        <v>45995.0</v>
+      </c>
+      <c r="M95" s="63">
+        <v>20000.0</v>
+      </c>
+      <c r="N95" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O95" s="66"/>
+      <c r="P95" s="67"/>
+      <c r="Q95" s="67"/>
+      <c r="R95" s="66"/>
+      <c r="S95" s="67"/>
+      <c r="T95" s="67"/>
+      <c r="U95" s="66"/>
+      <c r="V95" s="67"/>
+      <c r="W95" s="67"/>
+      <c r="X95" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y95" s="63" t="s">
+        <v>741</v>
+      </c>
+      <c r="Z95" s="63" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA95" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="AB95" s="62">
+        <v>3500.0</v>
+      </c>
+      <c r="AC95" s="63" t="s">
+        <v>921</v>
+      </c>
+      <c r="AD95" s="63" t="s">
+        <v>922</v>
+      </c>
+      <c r="AE95" s="63">
+        <v>9.198354186E9</v>
+      </c>
+      <c r="AF95" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG95" s="62">
+        <v>15.0</v>
+      </c>
+      <c r="AH95" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI95" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="62">
+        <v>652.0</v>
+      </c>
+      <c r="B96" s="63" t="s">
+        <v>279</v>
+      </c>
+      <c r="C96" s="64">
+        <v>45997.0</v>
+      </c>
+      <c r="D96" s="63" t="s">
+        <v>280</v>
+      </c>
+      <c r="E96" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F96" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G96" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H96" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I96" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J96" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K96" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L96" s="64">
+        <v>45997.0</v>
+      </c>
+      <c r="M96" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N96" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O96" s="66"/>
+      <c r="P96" s="67"/>
+      <c r="Q96" s="67"/>
+      <c r="R96" s="66"/>
+      <c r="S96" s="67"/>
+      <c r="T96" s="67"/>
+      <c r="U96" s="66"/>
+      <c r="V96" s="67"/>
+      <c r="W96" s="67"/>
+      <c r="X96" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y96" s="63" t="s">
+        <v>923</v>
+      </c>
+      <c r="Z96" s="63" t="s">
+        <v>924</v>
+      </c>
+      <c r="AA96" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB96" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC96" s="63" t="s">
+        <v>925</v>
+      </c>
+      <c r="AD96" s="63" t="s">
+        <v>926</v>
+      </c>
+      <c r="AE96" s="63">
+        <v>7.309853013E9</v>
+      </c>
+      <c r="AF96" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG96" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH96" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI96" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="62">
+        <v>708.0</v>
+      </c>
+      <c r="B97" s="63" t="s">
+        <v>284</v>
+      </c>
+      <c r="C97" s="64">
+        <v>46007.0</v>
+      </c>
+      <c r="D97" s="63" t="s">
+        <v>285</v>
+      </c>
+      <c r="E97" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F97" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G97" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H97" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I97" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J97" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K97" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L97" s="64">
+        <v>46007.0</v>
+      </c>
+      <c r="M97" s="63">
+        <v>8000.0</v>
+      </c>
+      <c r="N97" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O97" s="66"/>
+      <c r="P97" s="67"/>
+      <c r="Q97" s="67"/>
+      <c r="R97" s="66"/>
+      <c r="S97" s="67"/>
+      <c r="T97" s="67"/>
+      <c r="U97" s="66"/>
+      <c r="V97" s="67"/>
+      <c r="W97" s="67"/>
+      <c r="X97" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y97" s="63" t="s">
+        <v>741</v>
+      </c>
+      <c r="Z97" s="63" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA97" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB97" s="62">
+        <v>5560.0</v>
+      </c>
+      <c r="AC97" s="63" t="s">
+        <v>927</v>
+      </c>
+      <c r="AD97" s="63" t="s">
+        <v>928</v>
+      </c>
+      <c r="AE97" s="63">
+        <v>9.554598314E9</v>
+      </c>
+      <c r="AF97" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG97" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH97" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI97" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="62">
+        <v>771.0</v>
+      </c>
+      <c r="B98" s="63" t="s">
+        <v>288</v>
+      </c>
+      <c r="C98" s="64">
+        <v>46017.0</v>
+      </c>
+      <c r="D98" s="63" t="s">
+        <v>289</v>
+      </c>
+      <c r="E98" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F98" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G98" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H98" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I98" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J98" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K98" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L98" s="64">
+        <v>46017.0</v>
+      </c>
+      <c r="M98" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N98" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O98" s="66"/>
+      <c r="P98" s="67"/>
+      <c r="Q98" s="67"/>
+      <c r="R98" s="66"/>
+      <c r="S98" s="67"/>
+      <c r="T98" s="67"/>
+      <c r="U98" s="66"/>
+      <c r="V98" s="67"/>
+      <c r="W98" s="67"/>
+      <c r="X98" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y98" s="63" t="s">
+        <v>729</v>
+      </c>
+      <c r="Z98" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA98" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB98" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC98" s="63" t="s">
+        <v>929</v>
+      </c>
+      <c r="AD98" s="63" t="s">
+        <v>930</v>
+      </c>
+      <c r="AE98" s="63">
+        <v>6.387086703E9</v>
+      </c>
+      <c r="AF98" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG98" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH98" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI98" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="62">
+        <v>852.0</v>
+      </c>
+      <c r="B99" s="63" t="s">
+        <v>292</v>
+      </c>
+      <c r="C99" s="64">
+        <v>46030.0</v>
+      </c>
+      <c r="D99" s="63" t="s">
+        <v>293</v>
+      </c>
+      <c r="E99" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F99" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G99" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H99" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I99" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J99" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K99" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L99" s="64">
+        <v>46030.0</v>
+      </c>
+      <c r="M99" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N99" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O99" s="66"/>
+      <c r="P99" s="67"/>
+      <c r="Q99" s="67"/>
+      <c r="R99" s="66"/>
+      <c r="S99" s="67"/>
+      <c r="T99" s="67"/>
+      <c r="U99" s="66"/>
+      <c r="V99" s="67"/>
+      <c r="W99" s="67"/>
+      <c r="X99" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y99" s="63" t="s">
+        <v>741</v>
+      </c>
+      <c r="Z99" s="63" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA99" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB99" s="62">
+        <v>4150.0</v>
+      </c>
+      <c r="AC99" s="63" t="s">
+        <v>931</v>
+      </c>
+      <c r="AD99" s="63" t="s">
+        <v>932</v>
+      </c>
+      <c r="AE99" s="63">
+        <v>8.756954643E9</v>
+      </c>
+      <c r="AF99" s="63" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG99" s="62">
+        <v>15.0</v>
+      </c>
+      <c r="AH99" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI99" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="73"/>
+      <c r="B100" s="63" t="s">
+        <v>310</v>
+      </c>
+      <c r="C100" s="64">
+        <v>45780.0</v>
+      </c>
+      <c r="D100" s="63" t="s">
+        <v>311</v>
+      </c>
+      <c r="E100" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F100" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G100" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H100" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I100" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J100" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K100" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L100" s="64">
+        <v>45780.0</v>
+      </c>
+      <c r="M100" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N100" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O100" s="66"/>
+      <c r="P100" s="67"/>
+      <c r="Q100" s="67"/>
+      <c r="R100" s="66"/>
+      <c r="S100" s="67"/>
+      <c r="T100" s="67"/>
+      <c r="U100" s="66"/>
+      <c r="V100" s="67"/>
+      <c r="W100" s="67"/>
+      <c r="X100" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y100" s="63" t="s">
+        <v>312</v>
+      </c>
+      <c r="Z100" s="67"/>
+      <c r="AA100" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB100" s="62">
+        <v>4200.0</v>
+      </c>
+      <c r="AC100" s="63" t="s">
+        <v>933</v>
+      </c>
+      <c r="AD100" s="63" t="s">
+        <v>934</v>
+      </c>
+      <c r="AE100" s="63">
+        <v>8.69629024E9</v>
+      </c>
+      <c r="AF100" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG100" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH100" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI100" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="73"/>
+      <c r="B101" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="C101" s="64">
+        <v>45787.0</v>
+      </c>
+      <c r="D101" s="63" t="s">
+        <v>327</v>
+      </c>
+      <c r="E101" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F101" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G101" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H101" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I101" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J101" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K101" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L101" s="64">
+        <v>45787.0</v>
+      </c>
+      <c r="M101" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N101" s="67"/>
+      <c r="O101" s="66"/>
+      <c r="P101" s="67"/>
+      <c r="Q101" s="67"/>
+      <c r="R101" s="66"/>
+      <c r="S101" s="67"/>
+      <c r="T101" s="67"/>
+      <c r="U101" s="66"/>
+      <c r="V101" s="67"/>
+      <c r="W101" s="67"/>
+      <c r="X101" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y101" s="63" t="s">
+        <v>312</v>
+      </c>
+      <c r="Z101" s="63" t="s">
+        <v>935</v>
+      </c>
+      <c r="AA101" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB101" s="62">
+        <v>4200.0</v>
+      </c>
+      <c r="AC101" s="63" t="s">
+        <v>936</v>
+      </c>
+      <c r="AD101" s="63" t="s">
+        <v>937</v>
+      </c>
+      <c r="AE101" s="63">
+        <v>9.351825629E9</v>
+      </c>
+      <c r="AF101" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG101" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH101" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI101" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="73"/>
+      <c r="B102" s="63" t="s">
+        <v>348</v>
+      </c>
+      <c r="C102" s="64">
+        <v>45822.0</v>
+      </c>
+      <c r="D102" s="63" t="s">
+        <v>349</v>
+      </c>
+      <c r="E102" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F102" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G102" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H102" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="I102" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J102" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K102" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L102" s="64">
+        <v>45822.0</v>
+      </c>
+      <c r="M102" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N102" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="O102" s="66"/>
+      <c r="P102" s="67"/>
+      <c r="Q102" s="67"/>
+      <c r="R102" s="66"/>
+      <c r="S102" s="67"/>
+      <c r="T102" s="67"/>
+      <c r="U102" s="66"/>
+      <c r="V102" s="67"/>
+      <c r="W102" s="67"/>
+      <c r="X102" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y102" s="63" t="s">
+        <v>727</v>
+      </c>
+      <c r="Z102" s="63" t="s">
+        <v>938</v>
+      </c>
+      <c r="AA102" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB102" s="62">
+        <v>4200.0</v>
+      </c>
+      <c r="AC102" s="63" t="s">
+        <v>939</v>
+      </c>
+      <c r="AD102" s="63" t="s">
+        <v>940</v>
+      </c>
+      <c r="AE102" s="63">
+        <v>7.851091595E9</v>
+      </c>
+      <c r="AF102" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG102" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH102" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI102" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="73"/>
+      <c r="B103" s="63" t="s">
+        <v>361</v>
+      </c>
+      <c r="C103" s="64">
+        <v>45831.0</v>
+      </c>
+      <c r="D103" s="63" t="s">
+        <v>362</v>
+      </c>
+      <c r="E103" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F103" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G103" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H103" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I103" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J103" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K103" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L103" s="64">
+        <v>45831.0</v>
+      </c>
+      <c r="M103" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N103" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O103" s="66"/>
+      <c r="P103" s="67"/>
+      <c r="Q103" s="67"/>
+      <c r="R103" s="66"/>
+      <c r="S103" s="67"/>
+      <c r="T103" s="67"/>
+      <c r="U103" s="66"/>
+      <c r="V103" s="67"/>
+      <c r="W103" s="67"/>
+      <c r="X103" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y103" s="63" t="s">
+        <v>855</v>
+      </c>
+      <c r="Z103" s="63" t="s">
+        <v>313</v>
+      </c>
+      <c r="AA103" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB103" s="62">
+        <v>4200.0</v>
+      </c>
+      <c r="AC103" s="63" t="s">
+        <v>941</v>
+      </c>
+      <c r="AD103" s="63" t="s">
+        <v>942</v>
+      </c>
+      <c r="AE103" s="63">
+        <v>7.665858115E9</v>
+      </c>
+      <c r="AF103" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG103" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH103" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI103" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="73"/>
+      <c r="B104" s="63" t="s">
+        <v>367</v>
+      </c>
+      <c r="C104" s="64">
+        <v>45833.0</v>
+      </c>
+      <c r="D104" s="63" t="s">
+        <v>368</v>
+      </c>
+      <c r="E104" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F104" s="62">
+        <v>13000.0</v>
+      </c>
+      <c r="G104" s="62">
+        <v>13000.0</v>
+      </c>
+      <c r="H104" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I104" s="62">
+        <v>13000.0</v>
+      </c>
+      <c r="J104" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K104" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L104" s="64">
+        <v>45833.0</v>
+      </c>
+      <c r="M104" s="62">
+        <v>13000.0</v>
+      </c>
+      <c r="N104" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O104" s="66"/>
+      <c r="P104" s="67"/>
+      <c r="Q104" s="67"/>
+      <c r="R104" s="66"/>
+      <c r="S104" s="67"/>
+      <c r="T104" s="67"/>
+      <c r="U104" s="66"/>
+      <c r="V104" s="67"/>
+      <c r="W104" s="67"/>
+      <c r="X104" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y104" s="63" t="s">
+        <v>855</v>
+      </c>
+      <c r="Z104" s="63" t="s">
+        <v>313</v>
+      </c>
+      <c r="AA104" s="62">
+        <v>13000.0</v>
+      </c>
+      <c r="AB104" s="62">
+        <v>4410.0</v>
+      </c>
+      <c r="AC104" s="63" t="s">
+        <v>943</v>
+      </c>
+      <c r="AD104" s="63" t="s">
+        <v>944</v>
+      </c>
+      <c r="AE104" s="63">
+        <v>9.352427326E9</v>
+      </c>
+      <c r="AF104" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG104" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH104" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI104" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="73"/>
+      <c r="B105" s="63" t="s">
+        <v>425</v>
+      </c>
+      <c r="C105" s="64">
+        <v>45890.0</v>
+      </c>
+      <c r="D105" s="63" t="s">
+        <v>426</v>
+      </c>
+      <c r="E105" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F105" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G105" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H105" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I105" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J105" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K105" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L105" s="64">
+        <v>45890.0</v>
+      </c>
+      <c r="M105" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N105" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O105" s="66"/>
+      <c r="P105" s="67"/>
+      <c r="Q105" s="67"/>
+      <c r="R105" s="66"/>
+      <c r="S105" s="67"/>
+      <c r="T105" s="67"/>
+      <c r="U105" s="66"/>
+      <c r="V105" s="67"/>
+      <c r="W105" s="67"/>
+      <c r="X105" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y105" s="63" t="s">
+        <v>746</v>
+      </c>
+      <c r="Z105" s="63" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA105" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB105" s="62">
+        <v>5300.0</v>
+      </c>
+      <c r="AC105" s="63" t="s">
+        <v>945</v>
+      </c>
+      <c r="AD105" s="63" t="s">
+        <v>946</v>
+      </c>
+      <c r="AE105" s="63">
+        <v>9.694707266E9</v>
+      </c>
+      <c r="AF105" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG105" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH105" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI105" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="73"/>
+      <c r="B106" s="63" t="s">
+        <v>435</v>
+      </c>
+      <c r="C106" s="64">
+        <v>45908.0</v>
+      </c>
+      <c r="D106" s="63" t="s">
+        <v>436</v>
+      </c>
+      <c r="E106" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F106" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G106" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H106" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I106" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J106" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K106" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L106" s="64">
+        <v>45908.0</v>
+      </c>
+      <c r="M106" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N106" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O106" s="66"/>
+      <c r="P106" s="67"/>
+      <c r="Q106" s="67"/>
+      <c r="R106" s="66"/>
+      <c r="S106" s="67"/>
+      <c r="T106" s="67"/>
+      <c r="U106" s="66"/>
+      <c r="V106" s="67"/>
+      <c r="W106" s="67"/>
+      <c r="X106" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y106" s="63" t="s">
+        <v>947</v>
+      </c>
+      <c r="Z106" s="63" t="s">
+        <v>440</v>
+      </c>
+      <c r="AA106" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB106" s="62">
+        <v>5300.0</v>
+      </c>
+      <c r="AC106" s="63" t="s">
+        <v>948</v>
+      </c>
+      <c r="AD106" s="63" t="s">
+        <v>949</v>
+      </c>
+      <c r="AE106" s="63">
+        <v>8.058054538E9</v>
+      </c>
+      <c r="AF106" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG106" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH106" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI106" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="73"/>
+      <c r="B107" s="63" t="s">
+        <v>438</v>
+      </c>
+      <c r="C107" s="64">
+        <v>45908.0</v>
+      </c>
+      <c r="D107" s="63" t="s">
+        <v>439</v>
+      </c>
+      <c r="E107" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F107" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="G107" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="H107" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I107" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="J107" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K107" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L107" s="64">
+        <v>45908.0</v>
+      </c>
+      <c r="M107" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="N107" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O107" s="66"/>
+      <c r="P107" s="67"/>
+      <c r="Q107" s="67"/>
+      <c r="R107" s="66"/>
+      <c r="S107" s="67"/>
+      <c r="T107" s="67"/>
+      <c r="U107" s="66"/>
+      <c r="V107" s="67"/>
+      <c r="W107" s="67"/>
+      <c r="X107" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y107" s="63" t="s">
+        <v>947</v>
+      </c>
+      <c r="Z107" s="63" t="s">
+        <v>440</v>
+      </c>
+      <c r="AA107" s="62">
+        <v>6000.0</v>
+      </c>
+      <c r="AB107" s="62">
+        <v>5300.0</v>
+      </c>
+      <c r="AC107" s="63" t="s">
+        <v>950</v>
+      </c>
+      <c r="AD107" s="63" t="s">
+        <v>951</v>
+      </c>
+      <c r="AE107" s="63">
+        <v>9.529989436E9</v>
+      </c>
+      <c r="AF107" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG107" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH107" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI107" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="73"/>
+      <c r="B108" s="63" t="s">
+        <v>458</v>
+      </c>
+      <c r="C108" s="64">
+        <v>45947.0</v>
+      </c>
+      <c r="D108" s="63" t="s">
+        <v>459</v>
+      </c>
+      <c r="E108" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F108" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G108" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H108" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I108" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J108" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K108" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L108" s="64">
+        <v>45947.0</v>
+      </c>
+      <c r="M108" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="N108" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O108" s="66"/>
+      <c r="P108" s="67"/>
+      <c r="Q108" s="67"/>
+      <c r="R108" s="66"/>
+      <c r="S108" s="67"/>
+      <c r="T108" s="67"/>
+      <c r="U108" s="66"/>
+      <c r="V108" s="67"/>
+      <c r="W108" s="67"/>
+      <c r="X108" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y108" s="63" t="s">
+        <v>312</v>
+      </c>
+      <c r="Z108" s="63" t="s">
+        <v>315</v>
+      </c>
+      <c r="AA108" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB108" s="62">
+        <v>4360.0</v>
+      </c>
+      <c r="AC108" s="63" t="s">
+        <v>952</v>
+      </c>
+      <c r="AD108" s="63" t="s">
+        <v>953</v>
+      </c>
+      <c r="AE108" s="63">
+        <v>9.785922472E9</v>
+      </c>
+      <c r="AF108" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG108" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH108" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI108" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="73"/>
+      <c r="B109" s="63" t="s">
+        <v>461</v>
+      </c>
+      <c r="C109" s="64">
+        <v>45948.0</v>
+      </c>
+      <c r="D109" s="63" t="s">
+        <v>462</v>
+      </c>
+      <c r="E109" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F109" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G109" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H109" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="I109" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J109" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K109" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L109" s="64">
+        <v>45948.0</v>
+      </c>
+      <c r="M109" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N109" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="O109" s="66"/>
+      <c r="P109" s="67"/>
+      <c r="Q109" s="67"/>
+      <c r="R109" s="66"/>
+      <c r="S109" s="67"/>
+      <c r="T109" s="67"/>
+      <c r="U109" s="66"/>
+      <c r="V109" s="67"/>
+      <c r="W109" s="67"/>
+      <c r="X109" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y109" s="63" t="s">
+        <v>746</v>
+      </c>
+      <c r="Z109" s="63" t="s">
+        <v>954</v>
+      </c>
+      <c r="AA109" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB109" s="62">
+        <v>3130.0</v>
+      </c>
+      <c r="AC109" s="63" t="s">
+        <v>955</v>
+      </c>
+      <c r="AD109" s="63" t="s">
+        <v>956</v>
+      </c>
+      <c r="AE109" s="63">
+        <v>9.257851859E9</v>
+      </c>
+      <c r="AF109" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG109" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH109" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI109" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="73"/>
+      <c r="B110" s="63" t="s">
+        <v>464</v>
+      </c>
+      <c r="C110" s="64">
+        <v>45953.0</v>
+      </c>
+      <c r="D110" s="63" t="s">
+        <v>465</v>
+      </c>
+      <c r="E110" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F110" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G110" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H110" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I110" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J110" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K110" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L110" s="64">
+        <v>45953.0</v>
+      </c>
+      <c r="M110" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="N110" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O110" s="66"/>
+      <c r="P110" s="67"/>
+      <c r="Q110" s="67"/>
+      <c r="R110" s="66"/>
+      <c r="S110" s="67"/>
+      <c r="T110" s="67"/>
+      <c r="U110" s="66"/>
+      <c r="V110" s="67"/>
+      <c r="W110" s="67"/>
+      <c r="X110" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y110" s="63" t="s">
+        <v>957</v>
+      </c>
+      <c r="Z110" s="63" t="s">
+        <v>452</v>
+      </c>
+      <c r="AA110" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB110" s="62">
+        <v>4900.0</v>
+      </c>
+      <c r="AC110" s="63" t="s">
+        <v>958</v>
+      </c>
+      <c r="AD110" s="63" t="s">
+        <v>959</v>
+      </c>
+      <c r="AE110" s="63">
+        <v>7.891832996E9</v>
+      </c>
+      <c r="AF110" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG110" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH110" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI110" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="73"/>
+      <c r="B111" s="63" t="s">
+        <v>466</v>
+      </c>
+      <c r="C111" s="64">
+        <v>45968.0</v>
+      </c>
+      <c r="D111" s="63" t="s">
+        <v>467</v>
+      </c>
+      <c r="E111" s="63" t="s">
+        <v>813</v>
+      </c>
+      <c r="F111" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="G111" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="H111" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I111" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="J111" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K111" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L111" s="64">
+        <v>45968.0</v>
+      </c>
+      <c r="M111" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="N111" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O111" s="66"/>
+      <c r="P111" s="67"/>
+      <c r="Q111" s="67"/>
+      <c r="R111" s="66"/>
+      <c r="S111" s="67"/>
+      <c r="T111" s="67"/>
+      <c r="U111" s="66"/>
+      <c r="V111" s="67"/>
+      <c r="W111" s="67"/>
+      <c r="X111" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y111" s="63" t="s">
+        <v>960</v>
+      </c>
+      <c r="Z111" s="63" t="s">
+        <v>961</v>
+      </c>
+      <c r="AA111" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="AB111" s="62">
+        <v>9480.0</v>
+      </c>
+      <c r="AC111" s="63" t="s">
+        <v>962</v>
+      </c>
+      <c r="AD111" s="63" t="s">
+        <v>963</v>
+      </c>
+      <c r="AE111" s="63">
+        <v>9.77213637E9</v>
+      </c>
+      <c r="AF111" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG111" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH111" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI111" s="65" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="73"/>
+      <c r="B112" s="63" t="s">
+        <v>470</v>
+      </c>
+      <c r="C112" s="64">
+        <v>45971.0</v>
+      </c>
+      <c r="D112" s="63" t="s">
+        <v>471</v>
+      </c>
+      <c r="E112" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F112" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G112" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H112" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I112" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J112" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K112" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L112" s="64">
+        <v>45971.0</v>
+      </c>
+      <c r="M112" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="N112" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O112" s="66"/>
+      <c r="P112" s="67"/>
+      <c r="Q112" s="67"/>
+      <c r="R112" s="66"/>
+      <c r="S112" s="67"/>
+      <c r="T112" s="67"/>
+      <c r="U112" s="66"/>
+      <c r="V112" s="67"/>
+      <c r="W112" s="67"/>
+      <c r="X112" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y112" s="63" t="s">
+        <v>747</v>
+      </c>
+      <c r="Z112" s="63" t="s">
+        <v>965</v>
+      </c>
+      <c r="AA112" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB112" s="62">
+        <v>3620.0</v>
+      </c>
+      <c r="AC112" s="63" t="s">
+        <v>966</v>
+      </c>
+      <c r="AD112" s="63" t="s">
+        <v>967</v>
+      </c>
+      <c r="AE112" s="63">
+        <v>9.001729055E9</v>
+      </c>
+      <c r="AF112" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG112" s="62">
+        <v>15.0</v>
+      </c>
+      <c r="AH112" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI112" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="73"/>
+      <c r="B113" s="63" t="s">
+        <v>474</v>
+      </c>
+      <c r="C113" s="64">
+        <v>45973.0</v>
+      </c>
+      <c r="D113" s="63" t="s">
+        <v>475</v>
+      </c>
+      <c r="E113" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F113" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G113" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H113" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I113" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J113" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K113" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L113" s="64">
+        <v>45973.0</v>
+      </c>
+      <c r="M113" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="N113" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O113" s="66"/>
+      <c r="P113" s="67"/>
+      <c r="Q113" s="67"/>
+      <c r="R113" s="66"/>
+      <c r="S113" s="67"/>
+      <c r="T113" s="67"/>
+      <c r="U113" s="66"/>
+      <c r="V113" s="67"/>
+      <c r="W113" s="67"/>
+      <c r="X113" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y113" s="63" t="s">
+        <v>957</v>
+      </c>
+      <c r="Z113" s="63" t="s">
+        <v>452</v>
+      </c>
+      <c r="AA113" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB113" s="62">
+        <v>4900.0</v>
+      </c>
+      <c r="AC113" s="63" t="s">
+        <v>968</v>
+      </c>
+      <c r="AD113" s="63" t="s">
+        <v>969</v>
+      </c>
+      <c r="AE113" s="63">
+        <v>8.38686854E9</v>
+      </c>
+      <c r="AF113" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG113" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH113" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI113" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="73"/>
+      <c r="B114" s="63" t="s">
+        <v>476</v>
+      </c>
+      <c r="C114" s="64">
+        <v>45990.0</v>
+      </c>
+      <c r="D114" s="63" t="s">
+        <v>477</v>
+      </c>
+      <c r="E114" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F114" s="62">
+        <v>9000.0</v>
+      </c>
+      <c r="G114" s="62">
+        <v>9000.0</v>
+      </c>
+      <c r="H114" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I114" s="62">
+        <v>9000.0</v>
+      </c>
+      <c r="J114" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K114" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L114" s="64">
+        <v>45990.0</v>
+      </c>
+      <c r="M114" s="62">
+        <v>9000.0</v>
+      </c>
+      <c r="N114" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O114" s="66"/>
+      <c r="P114" s="67"/>
+      <c r="Q114" s="67"/>
+      <c r="R114" s="66"/>
+      <c r="S114" s="67"/>
+      <c r="T114" s="67"/>
+      <c r="U114" s="66"/>
+      <c r="V114" s="67"/>
+      <c r="W114" s="67"/>
+      <c r="X114" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y114" s="63" t="s">
+        <v>746</v>
+      </c>
+      <c r="Z114" s="63" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA114" s="62">
+        <v>9000.0</v>
+      </c>
+      <c r="AB114" s="62">
+        <v>3800.0</v>
+      </c>
+      <c r="AC114" s="63" t="s">
+        <v>970</v>
+      </c>
+      <c r="AD114" s="63" t="s">
+        <v>971</v>
+      </c>
+      <c r="AE114" s="63">
+        <v>9.251611573E9</v>
+      </c>
+      <c r="AF114" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG114" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH114" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI114" s="68"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="73"/>
+      <c r="B115" s="63" t="s">
+        <v>482</v>
+      </c>
+      <c r="C115" s="64">
+        <v>45995.0</v>
+      </c>
+      <c r="D115" s="63" t="s">
+        <v>483</v>
+      </c>
+      <c r="E115" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F115" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="G115" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="H115" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I115" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="J115" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K115" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L115" s="64">
+        <v>45995.0</v>
+      </c>
+      <c r="M115" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="N115" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O115" s="66"/>
+      <c r="P115" s="67"/>
+      <c r="Q115" s="67"/>
+      <c r="R115" s="66"/>
+      <c r="S115" s="67"/>
+      <c r="T115" s="67"/>
+      <c r="U115" s="66"/>
+      <c r="V115" s="67"/>
+      <c r="W115" s="67"/>
+      <c r="X115" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y115" s="63" t="s">
+        <v>957</v>
+      </c>
+      <c r="Z115" s="63" t="s">
+        <v>452</v>
+      </c>
+      <c r="AA115" s="62">
+        <v>8000.0</v>
+      </c>
+      <c r="AB115" s="62">
+        <v>5048.0</v>
+      </c>
+      <c r="AC115" s="63" t="s">
+        <v>972</v>
+      </c>
+      <c r="AD115" s="63" t="s">
+        <v>973</v>
+      </c>
+      <c r="AE115" s="63">
+        <v>6.350182421E9</v>
+      </c>
+      <c r="AF115" s="63" t="s">
+        <v>301</v>
+      </c>
+      <c r="AG115" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH115" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI115" s="68"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="62">
+        <v>114.0</v>
+      </c>
+      <c r="B116" s="63" t="s">
+        <v>551</v>
+      </c>
+      <c r="C116" s="64">
+        <v>45738.0</v>
+      </c>
+      <c r="D116" s="63" t="s">
+        <v>552</v>
+      </c>
+      <c r="E116" s="63" t="s">
+        <v>828</v>
+      </c>
+      <c r="F116" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="G116" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="H116" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I116" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="J116" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K116" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L116" s="64">
+        <v>45738.0</v>
+      </c>
+      <c r="M116" s="63">
+        <v>15000.0</v>
+      </c>
+      <c r="N116" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O116" s="66"/>
+      <c r="P116" s="67"/>
+      <c r="Q116" s="67"/>
+      <c r="R116" s="66"/>
+      <c r="S116" s="67"/>
+      <c r="T116" s="67"/>
+      <c r="U116" s="66"/>
+      <c r="V116" s="67"/>
+      <c r="W116" s="67"/>
+      <c r="X116" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y116" s="63" t="s">
+        <v>974</v>
+      </c>
+      <c r="Z116" s="67"/>
+      <c r="AA116" s="62">
+        <v>15000.0</v>
+      </c>
+      <c r="AB116" s="62">
+        <v>4560.0</v>
+      </c>
+      <c r="AC116" s="63" t="s">
+        <v>975</v>
+      </c>
+      <c r="AD116" s="63" t="s">
+        <v>976</v>
+      </c>
+      <c r="AE116" s="63">
+        <v>9.817002514E9</v>
+      </c>
+      <c r="AF116" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG116" s="63">
+        <v>18.0</v>
+      </c>
+      <c r="AH116" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI116" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="62">
+        <v>344.0</v>
+      </c>
+      <c r="B117" s="63" t="s">
+        <v>608</v>
+      </c>
+      <c r="C117" s="64">
+        <v>45873.0</v>
+      </c>
+      <c r="D117" s="63" t="s">
+        <v>609</v>
+      </c>
+      <c r="E117" s="63" t="s">
+        <v>813</v>
+      </c>
+      <c r="F117" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="G117" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="H117" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="I117" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="J117" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K117" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L117" s="64">
+        <v>45873.0</v>
+      </c>
+      <c r="M117" s="63">
+        <v>20000.0</v>
+      </c>
+      <c r="N117" s="63">
+        <v>5000.0</v>
+      </c>
+      <c r="O117" s="66"/>
+      <c r="P117" s="67"/>
+      <c r="Q117" s="67"/>
+      <c r="R117" s="66"/>
+      <c r="S117" s="67"/>
+      <c r="T117" s="67"/>
+      <c r="U117" s="66"/>
+      <c r="V117" s="67"/>
+      <c r="W117" s="67"/>
+      <c r="X117" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y117" s="63" t="s">
+        <v>753</v>
+      </c>
+      <c r="Z117" s="63" t="s">
+        <v>977</v>
+      </c>
+      <c r="AA117" s="62">
+        <v>25000.0</v>
+      </c>
+      <c r="AB117" s="62">
+        <v>7900.0</v>
+      </c>
+      <c r="AC117" s="63" t="s">
+        <v>978</v>
+      </c>
+      <c r="AD117" s="63" t="s">
+        <v>979</v>
+      </c>
+      <c r="AE117" s="63">
+        <v>8.396852271E9</v>
+      </c>
+      <c r="AF117" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG117" s="62">
+        <v>24.0</v>
+      </c>
+      <c r="AH117" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI117" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="62">
+        <v>387.0</v>
+      </c>
+      <c r="B118" s="63" t="s">
+        <v>620</v>
+      </c>
+      <c r="C118" s="64">
+        <v>45895.0</v>
+      </c>
+      <c r="D118" s="63" t="s">
+        <v>621</v>
+      </c>
+      <c r="E118" s="63" t="s">
+        <v>813</v>
+      </c>
+      <c r="F118" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="G118" s="62">
+        <v>16000.0</v>
+      </c>
+      <c r="H118" s="62">
+        <v>4000.0</v>
+      </c>
+      <c r="I118" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="J118" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K118" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L118" s="64">
+        <v>45895.0</v>
+      </c>
+      <c r="M118" s="63">
+        <v>16000.0</v>
+      </c>
+      <c r="N118" s="63">
+        <v>4000.0</v>
+      </c>
+      <c r="O118" s="66"/>
+      <c r="P118" s="67"/>
+      <c r="Q118" s="67"/>
+      <c r="R118" s="66"/>
+      <c r="S118" s="67"/>
+      <c r="T118" s="67"/>
+      <c r="U118" s="66"/>
+      <c r="V118" s="67"/>
+      <c r="W118" s="67"/>
+      <c r="X118" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y118" s="63" t="s">
+        <v>753</v>
+      </c>
+      <c r="Z118" s="63" t="s">
+        <v>980</v>
+      </c>
+      <c r="AA118" s="62">
+        <v>20000.0</v>
+      </c>
+      <c r="AB118" s="62">
+        <v>7900.0</v>
+      </c>
+      <c r="AC118" s="63" t="s">
+        <v>981</v>
+      </c>
+      <c r="AD118" s="63" t="s">
+        <v>982</v>
+      </c>
+      <c r="AE118" s="63">
+        <v>9.58818758E9</v>
+      </c>
+      <c r="AF118" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG118" s="62">
+        <v>24.0</v>
+      </c>
+      <c r="AH118" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI118" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="62">
+        <v>424.0</v>
+      </c>
+      <c r="B119" s="63" t="s">
+        <v>628</v>
+      </c>
+      <c r="C119" s="64">
+        <v>45905.0</v>
+      </c>
+      <c r="D119" s="63" t="s">
+        <v>528</v>
+      </c>
+      <c r="E119" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F119" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G119" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H119" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I119" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J119" s="62">
+        <v>4.0</v>
+      </c>
+      <c r="K119" s="65" t="s">
+        <v>983</v>
+      </c>
+      <c r="L119" s="64">
+        <v>45905.0</v>
+      </c>
+      <c r="M119" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N119" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O119" s="66"/>
+      <c r="P119" s="67"/>
+      <c r="Q119" s="67"/>
+      <c r="R119" s="66"/>
+      <c r="S119" s="67"/>
+      <c r="T119" s="67"/>
+      <c r="U119" s="66"/>
+      <c r="V119" s="67"/>
+      <c r="W119" s="67"/>
+      <c r="X119" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y119" s="63" t="s">
+        <v>494</v>
+      </c>
+      <c r="Z119" s="63" t="s">
+        <v>984</v>
+      </c>
+      <c r="AA119" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB119" s="62">
+        <v>3600.0</v>
+      </c>
+      <c r="AC119" s="63" t="s">
+        <v>985</v>
+      </c>
+      <c r="AD119" s="63" t="s">
+        <v>986</v>
+      </c>
+      <c r="AE119" s="63">
+        <v>8.168313221E9</v>
+      </c>
+      <c r="AF119" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG119" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH119" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI119" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="62">
+        <v>511.0</v>
+      </c>
+      <c r="B120" s="63" t="s">
+        <v>632</v>
+      </c>
+      <c r="C120" s="64">
+        <v>45934.0</v>
+      </c>
+      <c r="D120" s="63" t="s">
+        <v>633</v>
+      </c>
+      <c r="E120" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F120" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G120" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H120" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I120" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J120" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K120" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L120" s="64">
+        <v>45934.0</v>
+      </c>
+      <c r="M120" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N120" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O120" s="66"/>
+      <c r="P120" s="67"/>
+      <c r="Q120" s="67"/>
+      <c r="R120" s="66"/>
+      <c r="S120" s="67"/>
+      <c r="T120" s="67"/>
+      <c r="U120" s="66"/>
+      <c r="V120" s="67"/>
+      <c r="W120" s="67"/>
+      <c r="X120" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y120" s="63" t="s">
+        <v>764</v>
+      </c>
+      <c r="Z120" s="63" t="s">
+        <v>634</v>
+      </c>
+      <c r="AA120" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB120" s="62">
+        <v>3600.0</v>
+      </c>
+      <c r="AC120" s="63" t="s">
+        <v>987</v>
+      </c>
+      <c r="AD120" s="63" t="s">
+        <v>988</v>
+      </c>
+      <c r="AE120" s="63">
+        <v>8.570944626E9</v>
+      </c>
+      <c r="AF120" s="63" t="s">
+        <v>530</v>
+      </c>
+      <c r="AG120" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH120" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI120" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="62">
+        <v>551.0</v>
+      </c>
+      <c r="B121" s="63" t="s">
+        <v>642</v>
+      </c>
+      <c r="C121" s="64">
+        <v>45946.0</v>
+      </c>
+      <c r="D121" s="63" t="s">
+        <v>643</v>
+      </c>
+      <c r="E121" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F121" s="62">
+        <v>18000.0</v>
+      </c>
+      <c r="G121" s="62">
+        <v>18000.0</v>
+      </c>
+      <c r="H121" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I121" s="62">
+        <v>18000.0</v>
+      </c>
+      <c r="J121" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K121" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L121" s="64">
+        <v>45946.0</v>
+      </c>
+      <c r="M121" s="63">
+        <v>5000.0</v>
+      </c>
+      <c r="N121" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O121" s="64">
+        <v>45947.0</v>
+      </c>
+      <c r="P121" s="63">
+        <v>13000.0</v>
+      </c>
+      <c r="Q121" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="R121" s="66"/>
+      <c r="S121" s="67"/>
+      <c r="T121" s="67"/>
+      <c r="U121" s="66"/>
+      <c r="V121" s="67"/>
+      <c r="W121" s="67"/>
+      <c r="X121" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y121" s="63" t="s">
+        <v>989</v>
+      </c>
+      <c r="Z121" s="63" t="s">
+        <v>990</v>
+      </c>
+      <c r="AA121" s="62">
+        <v>18000.0</v>
+      </c>
+      <c r="AB121" s="62">
+        <v>3800.0</v>
+      </c>
+      <c r="AC121" s="63" t="s">
+        <v>991</v>
+      </c>
+      <c r="AD121" s="63" t="s">
+        <v>992</v>
+      </c>
+      <c r="AE121" s="63">
+        <v>9.728713204E9</v>
+      </c>
+      <c r="AF121" s="63" t="s">
+        <v>584</v>
+      </c>
+      <c r="AG121" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH121" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI121" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="62">
+        <v>598.0</v>
+      </c>
+      <c r="B122" s="63" t="s">
+        <v>654</v>
+      </c>
+      <c r="C122" s="64">
+        <v>45958.0</v>
+      </c>
+      <c r="D122" s="63" t="s">
+        <v>655</v>
+      </c>
+      <c r="E122" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F122" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G122" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H122" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="I122" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J122" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K122" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L122" s="64">
+        <v>45958.0</v>
+      </c>
+      <c r="M122" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N122" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="O122" s="66"/>
+      <c r="P122" s="67"/>
+      <c r="Q122" s="67"/>
+      <c r="R122" s="66"/>
+      <c r="S122" s="67"/>
+      <c r="T122" s="67"/>
+      <c r="U122" s="66"/>
+      <c r="V122" s="67"/>
+      <c r="W122" s="67"/>
+      <c r="X122" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y122" s="63" t="s">
+        <v>494</v>
+      </c>
+      <c r="Z122" s="63" t="s">
+        <v>993</v>
+      </c>
+      <c r="AA122" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB122" s="62">
+        <v>3600.0</v>
+      </c>
+      <c r="AC122" s="63" t="s">
+        <v>994</v>
+      </c>
+      <c r="AD122" s="63" t="s">
+        <v>995</v>
+      </c>
+      <c r="AE122" s="63">
+        <v>8.708651725E9</v>
+      </c>
+      <c r="AF122" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG122" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH122" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI122" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="62">
+        <v>640.0</v>
+      </c>
+      <c r="B123" s="63" t="s">
+        <v>658</v>
+      </c>
+      <c r="C123" s="64">
+        <v>45965.0</v>
+      </c>
+      <c r="D123" s="63" t="s">
+        <v>659</v>
+      </c>
+      <c r="E123" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F123" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G123" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H123" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I123" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J123" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K123" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L123" s="64">
+        <v>45965.0</v>
+      </c>
+      <c r="M123" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N123" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O123" s="66"/>
+      <c r="P123" s="67"/>
+      <c r="Q123" s="67"/>
+      <c r="R123" s="66"/>
+      <c r="S123" s="67"/>
+      <c r="T123" s="67"/>
+      <c r="U123" s="66"/>
+      <c r="V123" s="67"/>
+      <c r="W123" s="67"/>
+      <c r="X123" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y123" s="63" t="s">
+        <v>809</v>
+      </c>
+      <c r="Z123" s="63" t="s">
+        <v>810</v>
+      </c>
+      <c r="AA123" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB123" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC123" s="63" t="s">
+        <v>996</v>
+      </c>
+      <c r="AD123" s="63" t="s">
+        <v>997</v>
+      </c>
+      <c r="AE123" s="63">
+        <v>9.802471591E9</v>
+      </c>
+      <c r="AF123" s="63" t="s">
+        <v>584</v>
+      </c>
+      <c r="AG123" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH123" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI123" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="62">
+        <v>653.0</v>
+      </c>
+      <c r="B124" s="63" t="s">
+        <v>670</v>
+      </c>
+      <c r="C124" s="64">
+        <v>45968.0</v>
+      </c>
+      <c r="D124" s="63" t="s">
+        <v>671</v>
+      </c>
+      <c r="E124" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F124" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G124" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H124" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I124" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J124" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K124" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L124" s="64">
+        <v>45968.0</v>
+      </c>
+      <c r="M124" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N124" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O124" s="66"/>
+      <c r="P124" s="67"/>
+      <c r="Q124" s="67"/>
+      <c r="R124" s="66"/>
+      <c r="S124" s="67"/>
+      <c r="T124" s="67"/>
+      <c r="U124" s="66"/>
+      <c r="V124" s="67"/>
+      <c r="W124" s="67"/>
+      <c r="X124" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y124" s="63" t="s">
+        <v>764</v>
+      </c>
+      <c r="Z124" s="63" t="s">
+        <v>634</v>
+      </c>
+      <c r="AA124" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB124" s="62">
+        <v>4150.0</v>
+      </c>
+      <c r="AC124" s="63" t="s">
+        <v>998</v>
+      </c>
+      <c r="AD124" s="63" t="s">
+        <v>999</v>
+      </c>
+      <c r="AE124" s="63">
+        <v>8.059456852E9</v>
+      </c>
+      <c r="AF124" s="63" t="s">
+        <v>530</v>
+      </c>
+      <c r="AG124" s="62">
+        <v>15.0</v>
+      </c>
+      <c r="AH124" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI124" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="62">
+        <v>688.0</v>
+      </c>
+      <c r="B125" s="63" t="s">
+        <v>675</v>
+      </c>
+      <c r="C125" s="64">
+        <v>45976.0</v>
+      </c>
+      <c r="D125" s="63" t="s">
+        <v>676</v>
+      </c>
+      <c r="E125" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F125" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G125" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H125" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I125" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J125" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K125" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L125" s="64">
+        <v>45976.0</v>
+      </c>
+      <c r="M125" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N125" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O125" s="66"/>
+      <c r="P125" s="67"/>
+      <c r="Q125" s="67"/>
+      <c r="R125" s="66"/>
+      <c r="S125" s="67"/>
+      <c r="T125" s="67"/>
+      <c r="U125" s="66"/>
+      <c r="V125" s="67"/>
+      <c r="W125" s="67"/>
+      <c r="X125" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y125" s="63" t="s">
+        <v>734</v>
+      </c>
+      <c r="Z125" s="63" t="s">
+        <v>1000</v>
+      </c>
+      <c r="AA125" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB125" s="62">
+        <v>4400.0</v>
+      </c>
+      <c r="AC125" s="63" t="s">
+        <v>1001</v>
+      </c>
+      <c r="AD125" s="63" t="s">
+        <v>1002</v>
+      </c>
+      <c r="AE125" s="63">
+        <v>7.983489114E9</v>
+      </c>
+      <c r="AF125" s="63" t="s">
+        <v>638</v>
+      </c>
+      <c r="AG125" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH125" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI125" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="62">
+        <v>818.0</v>
+      </c>
+      <c r="B126" s="63" t="s">
+        <v>689</v>
+      </c>
+      <c r="C126" s="64">
+        <v>46014.0</v>
+      </c>
+      <c r="D126" s="63" t="s">
+        <v>690</v>
+      </c>
+      <c r="E126" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F126" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G126" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="H126" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I126" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J126" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K126" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L126" s="64">
+        <v>46014.0</v>
+      </c>
+      <c r="M126" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="N126" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O126" s="66"/>
+      <c r="P126" s="67"/>
+      <c r="Q126" s="67"/>
+      <c r="R126" s="66"/>
+      <c r="S126" s="67"/>
+      <c r="T126" s="67"/>
+      <c r="U126" s="66"/>
+      <c r="V126" s="67"/>
+      <c r="W126" s="67"/>
+      <c r="X126" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y126" s="63" t="s">
+        <v>734</v>
+      </c>
+      <c r="Z126" s="63" t="s">
+        <v>806</v>
+      </c>
+      <c r="AA126" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB126" s="62">
+        <v>3020.0</v>
+      </c>
+      <c r="AC126" s="63" t="s">
+        <v>1003</v>
+      </c>
+      <c r="AD126" s="63" t="s">
+        <v>1004</v>
+      </c>
+      <c r="AE126" s="63">
+        <v>7.535028703E9</v>
+      </c>
+      <c r="AF126" s="63" t="s">
+        <v>638</v>
+      </c>
+      <c r="AG126" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH126" s="65" t="s">
+        <v>769</v>
+      </c>
+      <c r="AI126" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="62">
+        <v>887.0</v>
+      </c>
+      <c r="B127" s="63" t="s">
+        <v>693</v>
+      </c>
+      <c r="C127" s="64">
+        <v>46008.0</v>
+      </c>
+      <c r="D127" s="63" t="s">
+        <v>694</v>
+      </c>
+      <c r="E127" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F127" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="G127" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H127" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="I127" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="J127" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K127" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L127" s="64">
+        <v>46008.0</v>
+      </c>
+      <c r="M127" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="N127" s="63">
+        <v>12000.0</v>
+      </c>
+      <c r="O127" s="66"/>
+      <c r="P127" s="67"/>
+      <c r="Q127" s="67"/>
+      <c r="R127" s="66"/>
+      <c r="S127" s="67"/>
+      <c r="T127" s="67"/>
+      <c r="U127" s="66"/>
+      <c r="V127" s="67"/>
+      <c r="W127" s="67"/>
+      <c r="X127" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y127" s="63" t="s">
+        <v>494</v>
+      </c>
+      <c r="Z127" s="63" t="s">
+        <v>1005</v>
+      </c>
+      <c r="AA127" s="62">
+        <v>12000.0</v>
+      </c>
+      <c r="AB127" s="62">
+        <v>5000.0</v>
+      </c>
+      <c r="AC127" s="63" t="s">
+        <v>1006</v>
+      </c>
+      <c r="AD127" s="63" t="s">
+        <v>1007</v>
+      </c>
+      <c r="AE127" s="63">
+        <v>9.46819126E9</v>
+      </c>
+      <c r="AF127" s="63" t="s">
+        <v>491</v>
+      </c>
+      <c r="AG127" s="62">
+        <v>12.0</v>
+      </c>
+      <c r="AH127" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI127" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="62">
+        <v>973.0</v>
+      </c>
+      <c r="B128" s="63" t="s">
+        <v>698</v>
+      </c>
+      <c r="C128" s="64">
+        <v>46042.0</v>
+      </c>
+      <c r="D128" s="63" t="s">
+        <v>699</v>
+      </c>
+      <c r="E128" s="63" t="s">
+        <v>749</v>
+      </c>
+      <c r="F128" s="62">
+        <v>10000.0</v>
+      </c>
+      <c r="G128" s="62">
+        <v>10000.0</v>
+      </c>
+      <c r="H128" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="I128" s="62">
+        <v>10000.0</v>
+      </c>
+      <c r="J128" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="K128" s="65" t="s">
+        <v>728</v>
+      </c>
+      <c r="L128" s="64">
+        <v>46042.0</v>
+      </c>
+      <c r="M128" s="63">
+        <v>10000.0</v>
+      </c>
+      <c r="N128" s="63">
+        <v>0.0</v>
+      </c>
+      <c r="O128" s="66"/>
+      <c r="P128" s="67"/>
+      <c r="Q128" s="67"/>
+      <c r="R128" s="66"/>
+      <c r="S128" s="67"/>
+      <c r="T128" s="67"/>
+      <c r="U128" s="66"/>
+      <c r="V128" s="67"/>
+      <c r="W128" s="67"/>
+      <c r="X128" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="Y128" s="63" t="s">
+        <v>734</v>
+      </c>
+      <c r="Z128" s="63" t="s">
+        <v>669</v>
+      </c>
+      <c r="AA128" s="62">
+        <v>10000.0</v>
+      </c>
+      <c r="AB128" s="62">
+        <v>3850.0</v>
+      </c>
+      <c r="AC128" s="63" t="s">
+        <v>1008</v>
+      </c>
+      <c r="AD128" s="63" t="s">
+        <v>1009</v>
+      </c>
+      <c r="AE128" s="63">
+        <v>9.045615011E9</v>
+      </c>
+      <c r="AF128" s="63" t="s">
+        <v>638</v>
+      </c>
+      <c r="AG128" s="62">
+        <v>18.0</v>
+      </c>
+      <c r="AH128" s="65" t="s">
+        <v>752</v>
+      </c>
+      <c r="AI128" s="65" t="s">
+        <v>728</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>